<commit_message>
update with aleix data
</commit_message>
<xml_diff>
--- a/05_screening/validation_screening.xlsx
+++ b/05_screening/validation_screening.xlsx
@@ -848,10 +848,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
-      <c r="L2" s="5" t="n"/>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -892,10 +908,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
-      <c r="L3" s="5" t="n"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -932,10 +964,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
-      <c r="L4" s="5" t="n"/>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -976,10 +1024,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
-      <c r="L5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -1020,10 +1084,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
-      <c r="L6" s="5" t="n"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -1060,10 +1140,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
@@ -1104,10 +1200,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
-      <c r="L8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -1148,10 +1260,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
@@ -1192,10 +1320,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -1236,10 +1380,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
@@ -1280,10 +1440,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="5" t="n"/>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -1324,10 +1500,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1368,10 +1560,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
-      <c r="L14" s="5" t="n"/>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -1412,10 +1620,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-      <c r="L15" s="5" t="n"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
@@ -1456,10 +1680,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
-      <c r="L16" s="5" t="n"/>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -1496,10 +1736,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
@@ -1540,10 +1796,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
-      <c r="L18" s="5" t="n"/>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
@@ -1584,10 +1856,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
@@ -1628,10 +1916,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
-      <c r="K20" s="5" t="n"/>
-      <c r="L20" s="5" t="n"/>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
@@ -1672,10 +1976,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-      <c r="L21" s="5" t="n"/>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
@@ -1712,10 +2032,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="5" t="n"/>
-      <c r="K22" s="5" t="n"/>
-      <c r="L22" s="5" t="n"/>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -1756,10 +2092,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
-      <c r="L23" s="5" t="n"/>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -1800,10 +2152,26 @@
           <t>semantic_scholar</t>
         </is>
       </c>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="5" t="n"/>
-      <c r="K24" s="5" t="n"/>
-      <c r="L24" s="5" t="n"/>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
@@ -1844,10 +2212,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="n"/>
-      <c r="K25" s="5" t="n"/>
-      <c r="L25" s="5" t="n"/>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="n">
@@ -1888,10 +2272,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="5" t="n"/>
-      <c r="K26" s="5" t="n"/>
-      <c r="L26" s="5" t="n"/>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -1932,10 +2332,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
-      <c r="K27" s="5" t="n"/>
-      <c r="L27" s="5" t="n"/>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -1976,10 +2392,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="5" t="n"/>
-      <c r="L28" s="5" t="n"/>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
@@ -2020,10 +2452,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="5" t="n"/>
-      <c r="K29" s="5" t="n"/>
-      <c r="L29" s="5" t="n"/>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="n">
@@ -2060,10 +2508,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="5" t="n"/>
-      <c r="L30" s="5" t="n"/>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
@@ -2100,10 +2564,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="5" t="n"/>
-      <c r="L31" s="5" t="n"/>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -2140,10 +2620,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I32" s="5" t="n"/>
-      <c r="J32" s="5" t="n"/>
-      <c r="K32" s="5" t="n"/>
-      <c r="L32" s="5" t="n"/>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -2184,10 +2680,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="n"/>
-      <c r="K33" s="5" t="n"/>
-      <c r="L33" s="5" t="n"/>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -2228,10 +2740,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I34" s="5" t="n"/>
-      <c r="J34" s="5" t="n"/>
-      <c r="K34" s="5" t="n"/>
-      <c r="L34" s="5" t="n"/>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -2272,10 +2800,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="5" t="n"/>
-      <c r="K35" s="5" t="n"/>
-      <c r="L35" s="5" t="n"/>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -2312,10 +2856,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="5" t="n"/>
-      <c r="L36" s="5" t="n"/>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -2352,10 +2912,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="n"/>
-      <c r="K37" s="5" t="n"/>
-      <c r="L37" s="5" t="n"/>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -2392,10 +2968,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="5" t="n"/>
-      <c r="K38" s="5" t="n"/>
-      <c r="L38" s="5" t="n"/>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -2432,10 +3024,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="5" t="n"/>
-      <c r="L39" s="5" t="n"/>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
@@ -2476,10 +3084,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
-      <c r="L40" s="5" t="n"/>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -2520,10 +3144,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="5" t="n"/>
-      <c r="L41" s="5" t="n"/>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="n">
@@ -2564,10 +3204,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="5" t="n"/>
-      <c r="K42" s="5" t="n"/>
-      <c r="L42" s="5" t="n"/>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K42" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="n">
@@ -2608,10 +3264,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I43" s="5" t="n"/>
-      <c r="J43" s="5" t="n"/>
-      <c r="K43" s="5" t="n"/>
-      <c r="L43" s="5" t="n"/>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -2652,10 +3324,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I44" s="5" t="n"/>
-      <c r="J44" s="5" t="n"/>
-      <c r="K44" s="5" t="n"/>
-      <c r="L44" s="5" t="n"/>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L44" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -2696,10 +3384,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I45" s="5" t="n"/>
-      <c r="J45" s="5" t="n"/>
-      <c r="K45" s="5" t="n"/>
-      <c r="L45" s="5" t="n"/>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L45" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -2740,10 +3444,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I46" s="5" t="n"/>
-      <c r="J46" s="5" t="n"/>
-      <c r="K46" s="5" t="n"/>
-      <c r="L46" s="5" t="n"/>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L46" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -2784,10 +3504,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I47" s="5" t="n"/>
-      <c r="J47" s="5" t="n"/>
-      <c r="K47" s="5" t="n"/>
-      <c r="L47" s="5" t="n"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="n">
@@ -2828,10 +3564,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I48" s="5" t="n"/>
-      <c r="J48" s="5" t="n"/>
-      <c r="K48" s="5" t="n"/>
-      <c r="L48" s="5" t="n"/>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L48" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="n">
@@ -2868,10 +3620,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I49" s="5" t="n"/>
-      <c r="J49" s="5" t="n"/>
-      <c r="K49" s="5" t="n"/>
-      <c r="L49" s="5" t="n"/>
+      <c r="I49" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L49" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="n">
@@ -2912,10 +3680,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I50" s="5" t="n"/>
-      <c r="J50" s="5" t="n"/>
-      <c r="K50" s="5" t="n"/>
-      <c r="L50" s="5" t="n"/>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -2952,10 +3736,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I51" s="5" t="n"/>
-      <c r="J51" s="5" t="n"/>
-      <c r="K51" s="5" t="n"/>
-      <c r="L51" s="5" t="n"/>
+      <c r="I51" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L51" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
@@ -2996,10 +3796,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I52" s="5" t="n"/>
-      <c r="J52" s="5" t="n"/>
-      <c r="K52" s="5" t="n"/>
-      <c r="L52" s="5" t="n"/>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -3040,10 +3856,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I53" s="5" t="n"/>
-      <c r="J53" s="5" t="n"/>
-      <c r="K53" s="5" t="n"/>
-      <c r="L53" s="5" t="n"/>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -3084,10 +3916,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I54" s="5" t="n"/>
-      <c r="J54" s="5" t="n"/>
-      <c r="K54" s="5" t="n"/>
-      <c r="L54" s="5" t="n"/>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
@@ -3124,10 +3972,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I55" s="5" t="n"/>
-      <c r="J55" s="5" t="n"/>
-      <c r="K55" s="5" t="n"/>
-      <c r="L55" s="5" t="n"/>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K55" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L55" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
@@ -3164,10 +4028,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I56" s="5" t="n"/>
-      <c r="J56" s="5" t="n"/>
-      <c r="K56" s="5" t="n"/>
-      <c r="L56" s="5" t="n"/>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K56" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L56" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="n">
@@ -3204,10 +4084,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I57" s="5" t="n"/>
-      <c r="J57" s="5" t="n"/>
-      <c r="K57" s="5" t="n"/>
-      <c r="L57" s="5" t="n"/>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n">
@@ -3248,10 +4144,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I58" s="5" t="n"/>
-      <c r="J58" s="5" t="n"/>
-      <c r="K58" s="5" t="n"/>
-      <c r="L58" s="5" t="n"/>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L58" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="n">
@@ -3288,10 +4200,26 @@
           <t>semantic_scholar</t>
         </is>
       </c>
-      <c r="I59" s="5" t="n"/>
-      <c r="J59" s="5" t="n"/>
-      <c r="K59" s="5" t="n"/>
-      <c r="L59" s="5" t="n"/>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K59" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -3332,10 +4260,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I60" s="5" t="n"/>
-      <c r="J60" s="5" t="n"/>
-      <c r="K60" s="5" t="n"/>
-      <c r="L60" s="5" t="n"/>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K60" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L60" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -3376,10 +4320,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I61" s="5" t="n"/>
-      <c r="J61" s="5" t="n"/>
-      <c r="K61" s="5" t="n"/>
-      <c r="L61" s="5" t="n"/>
+      <c r="I61" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -3420,10 +4380,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I62" s="5" t="n"/>
-      <c r="J62" s="5" t="n"/>
-      <c r="K62" s="5" t="n"/>
-      <c r="L62" s="5" t="n"/>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K62" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L62" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -3464,10 +4440,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I63" s="5" t="n"/>
-      <c r="J63" s="5" t="n"/>
-      <c r="K63" s="5" t="n"/>
-      <c r="L63" s="5" t="n"/>
+      <c r="I63" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K63" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L63" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -3496,10 +4488,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I64" s="5" t="n"/>
-      <c r="J64" s="5" t="n"/>
-      <c r="K64" s="5" t="n"/>
-      <c r="L64" s="5" t="n"/>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K64" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
@@ -3536,10 +4544,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I65" s="5" t="n"/>
-      <c r="J65" s="5" t="n"/>
-      <c r="K65" s="5" t="n"/>
-      <c r="L65" s="5" t="n"/>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K65" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L65" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
@@ -3576,10 +4600,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I66" s="5" t="n"/>
-      <c r="J66" s="5" t="n"/>
-      <c r="K66" s="5" t="n"/>
-      <c r="L66" s="5" t="n"/>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n">
@@ -3620,10 +4660,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I67" s="5" t="n"/>
-      <c r="J67" s="5" t="n"/>
-      <c r="K67" s="5" t="n"/>
-      <c r="L67" s="5" t="n"/>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="n">
@@ -3664,10 +4720,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I68" s="5" t="n"/>
-      <c r="J68" s="5" t="n"/>
-      <c r="K68" s="5" t="n"/>
-      <c r="L68" s="5" t="n"/>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K68" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n">
@@ -3704,10 +4776,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I69" s="5" t="n"/>
-      <c r="J69" s="5" t="n"/>
-      <c r="K69" s="5" t="n"/>
-      <c r="L69" s="5" t="n"/>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="n">
@@ -3744,10 +4832,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I70" s="5" t="n"/>
-      <c r="J70" s="5" t="n"/>
-      <c r="K70" s="5" t="n"/>
-      <c r="L70" s="5" t="n"/>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K70" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L70" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n">
@@ -3784,10 +4888,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I71" s="5" t="n"/>
-      <c r="J71" s="5" t="n"/>
-      <c r="K71" s="5" t="n"/>
-      <c r="L71" s="5" t="n"/>
+      <c r="I71" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L71" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -3824,10 +4944,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I72" s="5" t="n"/>
-      <c r="J72" s="5" t="n"/>
-      <c r="K72" s="5" t="n"/>
-      <c r="L72" s="5" t="n"/>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L72" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="n">
@@ -3868,10 +5004,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I73" s="5" t="n"/>
-      <c r="J73" s="5" t="n"/>
-      <c r="K73" s="5" t="n"/>
-      <c r="L73" s="5" t="n"/>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L73" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="n">
@@ -3908,10 +5060,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I74" s="5" t="n"/>
-      <c r="J74" s="5" t="n"/>
-      <c r="K74" s="5" t="n"/>
-      <c r="L74" s="5" t="n"/>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L74" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n">
@@ -3952,10 +5120,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I75" s="5" t="n"/>
-      <c r="J75" s="5" t="n"/>
-      <c r="K75" s="5" t="n"/>
-      <c r="L75" s="5" t="n"/>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L75" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="n">
@@ -3992,10 +5176,26 @@
           <t>semantic_scholar</t>
         </is>
       </c>
-      <c r="I76" s="5" t="n"/>
-      <c r="J76" s="5" t="n"/>
-      <c r="K76" s="5" t="n"/>
-      <c r="L76" s="5" t="n"/>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="n">
@@ -4036,10 +5236,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I77" s="5" t="n"/>
-      <c r="J77" s="5" t="n"/>
-      <c r="K77" s="5" t="n"/>
-      <c r="L77" s="5" t="n"/>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K77" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L77" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
@@ -4080,10 +5296,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I78" s="5" t="n"/>
-      <c r="J78" s="5" t="n"/>
-      <c r="K78" s="5" t="n"/>
-      <c r="L78" s="5" t="n"/>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L78" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="n">
@@ -4124,10 +5356,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I79" s="5" t="n"/>
-      <c r="J79" s="5" t="n"/>
-      <c r="K79" s="5" t="n"/>
-      <c r="L79" s="5" t="n"/>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K79" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L79" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="n">
@@ -4168,10 +5416,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I80" s="5" t="n"/>
-      <c r="J80" s="5" t="n"/>
-      <c r="K80" s="5" t="n"/>
-      <c r="L80" s="5" t="n"/>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L80" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="n">
@@ -4212,10 +5476,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I81" s="5" t="n"/>
-      <c r="J81" s="5" t="n"/>
-      <c r="K81" s="5" t="n"/>
-      <c r="L81" s="5" t="n"/>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K81" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L81" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
@@ -4256,10 +5536,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I82" s="5" t="n"/>
-      <c r="J82" s="5" t="n"/>
-      <c r="K82" s="5" t="n"/>
-      <c r="L82" s="5" t="n"/>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L82" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n">
@@ -4300,10 +5596,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I83" s="5" t="n"/>
-      <c r="J83" s="5" t="n"/>
-      <c r="K83" s="5" t="n"/>
-      <c r="L83" s="5" t="n"/>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K83" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L83" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
@@ -4340,10 +5652,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I84" s="5" t="n"/>
-      <c r="J84" s="5" t="n"/>
-      <c r="K84" s="5" t="n"/>
-      <c r="L84" s="5" t="n"/>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K84" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L84" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n">
@@ -4384,10 +5712,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I85" s="5" t="n"/>
-      <c r="J85" s="5" t="n"/>
-      <c r="K85" s="5" t="n"/>
-      <c r="L85" s="5" t="n"/>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K85" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L85" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n">
@@ -4420,10 +5764,26 @@
           <t>scopus</t>
         </is>
       </c>
-      <c r="I86" s="5" t="n"/>
-      <c r="J86" s="5" t="n"/>
-      <c r="K86" s="5" t="n"/>
-      <c r="L86" s="5" t="n"/>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L86" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n">
@@ -4464,10 +5824,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I87" s="5" t="n"/>
-      <c r="J87" s="5" t="n"/>
-      <c r="K87" s="5" t="n"/>
-      <c r="L87" s="5" t="n"/>
+      <c r="I87" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K87" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L87" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="n">
@@ -4508,10 +5884,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I88" s="5" t="n"/>
-      <c r="J88" s="5" t="n"/>
-      <c r="K88" s="5" t="n"/>
-      <c r="L88" s="5" t="n"/>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K88" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L88" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="n">
@@ -4548,10 +5940,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I89" s="5" t="n"/>
-      <c r="J89" s="5" t="n"/>
-      <c r="K89" s="5" t="n"/>
-      <c r="L89" s="5" t="n"/>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J89" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K89" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L89" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="n">
@@ -4592,10 +6000,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I90" s="5" t="n"/>
-      <c r="J90" s="5" t="n"/>
-      <c r="K90" s="5" t="n"/>
-      <c r="L90" s="5" t="n"/>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K90" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L90" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="n">
@@ -4632,10 +6056,26 @@
           <t>semantic_scholar</t>
         </is>
       </c>
-      <c r="I91" s="5" t="n"/>
-      <c r="J91" s="5" t="n"/>
-      <c r="K91" s="5" t="n"/>
-      <c r="L91" s="5" t="n"/>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J91" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K91" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L91" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="n">
@@ -4676,10 +6116,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I92" s="5" t="n"/>
-      <c r="J92" s="5" t="n"/>
-      <c r="K92" s="5" t="n"/>
-      <c r="L92" s="5" t="n"/>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K92" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L92" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="n">
@@ -4720,10 +6176,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I93" s="5" t="n"/>
-      <c r="J93" s="5" t="n"/>
-      <c r="K93" s="5" t="n"/>
-      <c r="L93" s="5" t="n"/>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K93" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L93" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n">
@@ -4764,10 +6236,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I94" s="5" t="n"/>
-      <c r="J94" s="5" t="n"/>
-      <c r="K94" s="5" t="n"/>
-      <c r="L94" s="5" t="n"/>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="K94" s="5" t="inlineStr">
+        <is>
+          <t>include</t>
+        </is>
+      </c>
+      <c r="L94" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="n">
@@ -4808,10 +6296,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I95" s="5" t="n"/>
-      <c r="J95" s="5" t="n"/>
-      <c r="K95" s="5" t="n"/>
-      <c r="L95" s="5" t="n"/>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J95" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K95" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L95" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="n">
@@ -4852,10 +6356,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I96" s="5" t="n"/>
-      <c r="J96" s="5" t="n"/>
-      <c r="K96" s="5" t="n"/>
-      <c r="L96" s="5" t="n"/>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J96" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K96" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L96" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="n">
@@ -4896,10 +6416,26 @@
           <t>openalex</t>
         </is>
       </c>
-      <c r="I97" s="5" t="n"/>
-      <c r="J97" s="5" t="n"/>
-      <c r="K97" s="5" t="n"/>
-      <c r="L97" s="5" t="n"/>
+      <c r="I97" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J97" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K97" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L97" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n">
@@ -4940,10 +6476,26 @@
           <t>arxiv</t>
         </is>
       </c>
-      <c r="I98" s="5" t="n"/>
-      <c r="J98" s="5" t="n"/>
-      <c r="K98" s="5" t="n"/>
-      <c r="L98" s="5" t="n"/>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J98" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K98" s="5" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L98" s="5" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4979,6 +6531,26 @@
           <t>arxiv</t>
         </is>
       </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -5019,6 +6591,26 @@
           <t>openalex</t>
         </is>
       </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -5054,6 +6646,26 @@
           <t>scopus</t>
         </is>
       </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -5092,6 +6704,26 @@
       <c r="H102" t="inlineStr">
         <is>
           <t>openalex</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>exclude</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>Filled from AI screening decisions</t>
         </is>
       </c>
     </row>

</xml_diff>